<commit_message>
Update DLS journal + dls.json
</commit_message>
<xml_diff>
--- a/data/Журнал_ДЛС.xlsx
+++ b/data/Журнал_ДЛС.xlsx
@@ -11143,7 +11143,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H18"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -11666,7 +11666,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>№ 434-001.001/002.0/17-26 від 11.09.2026</t>
+          <t>№ 434-001.001/002.0 17-26 від 11.09.2026</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -11676,7 +11676,7 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>DYSPORT® 500 U (Botulinum toxin type A), ліофілізований порошок, Серія № P08193, з маркуванням Ipsen Farmaceutica Ltda, -</t>
+          <t>СТРЕПСІЛС® З ВІТАМІНОМ С ЗІ СМАКОМ АПЕЛЬСИНА, льодяники, по 12 льодяників у блістері; по 2 блістери в картонній коробці, Серія № ST420, Реккітт Бенкізер Хелскер Інтернешнл Лімітед, Велика Британiя</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
@@ -11687,6 +11687,34 @@
       <c r="F18" s="2" t="inlineStr"/>
       <c r="G18" s="2" t="inlineStr"/>
       <c r="H18" s="2" t="inlineStr"/>
+    </row>
+    <row r="19" ht="40" customHeight="1">
+      <c r="A19" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>№ 434-001.001/002.0/17-26 від 11.09.2026</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>11.09.2026</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>DYSPORT® 500 U (Botulinum toxin type A), ліофілізований порошок, Серія № P08193, з маркуванням Ipsen Farmaceutica Ltda, -</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>відсутній</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr"/>
+      <c r="G19" s="2" t="inlineStr"/>
+      <c r="H19" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>